<commit_message>
10orders instant manufacture and 100orders solution1
10order的整理了下，在cp框架下添加实现了立即生产的相关约束，100order的之前没commit这次整理了下一起传了
</commit_message>
<xml_diff>
--- a/steel_fabucation_arrangement/solution/lirui/schedule_sol_sheet_数据1_exact.xlsx
+++ b/steel_fabucation_arrangement/solution/lirui/schedule_sol_sheet_数据1_exact.xlsx
@@ -503,37 +503,37 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>600</v>
+        <v>878</v>
       </c>
       <c r="D2" t="n">
-        <v>1212</v>
+        <v>1490</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>1481</v>
+        <v>1490</v>
       </c>
       <c r="G2" t="n">
-        <v>2023</v>
+        <v>2032</v>
       </c>
       <c r="H2" t="n">
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>2023</v>
+        <v>2032</v>
       </c>
       <c r="J2" t="n">
-        <v>2809</v>
+        <v>2818</v>
       </c>
       <c r="K2" t="n">
         <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>2809</v>
+        <v>2818</v>
       </c>
       <c r="M2" t="n">
-        <v>3002</v>
+        <v>3011</v>
       </c>
     </row>
     <row r="3">
@@ -541,13 +541,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1881</v>
+        <v>2345</v>
       </c>
       <c r="D3" t="n">
-        <v>2302</v>
+        <v>2634</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -582,40 +582,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>2302</v>
+        <v>1844</v>
       </c>
       <c r="D4" t="n">
-        <v>2636</v>
+        <v>2345</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>2819</v>
+        <v>2828</v>
       </c>
       <c r="G4" t="n">
-        <v>3647</v>
+        <v>3656</v>
       </c>
       <c r="H4" t="n">
         <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>3687</v>
+        <v>3696</v>
       </c>
       <c r="J4" t="n">
-        <v>4024</v>
+        <v>4033</v>
       </c>
       <c r="K4" t="n">
         <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>4024</v>
+        <v>4033</v>
       </c>
       <c r="M4" t="n">
-        <v>4136</v>
+        <v>4145</v>
       </c>
     </row>
     <row r="5">
@@ -623,13 +623,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>766</v>
+        <v>600</v>
       </c>
       <c r="D5" t="n">
-        <v>1389</v>
+        <v>878</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -644,19 +644,19 @@
         <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>2809</v>
+        <v>2818</v>
       </c>
       <c r="J5" t="n">
-        <v>3289</v>
+        <v>3298</v>
       </c>
       <c r="K5" t="n">
         <v>2</v>
       </c>
       <c r="L5" t="n">
-        <v>3289</v>
+        <v>3298</v>
       </c>
       <c r="M5" t="n">
-        <v>3668</v>
+        <v>3677</v>
       </c>
     </row>
     <row r="6">
@@ -667,10 +667,10 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D6" t="n">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -685,19 +685,19 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1498</v>
+        <v>1565</v>
       </c>
       <c r="J6" t="n">
-        <v>2033</v>
+        <v>2100</v>
       </c>
       <c r="K6" t="n">
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>2033</v>
+        <v>2100</v>
       </c>
       <c r="M6" t="n">
-        <v>2492</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="7">
@@ -705,40 +705,40 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>1214</v>
+        <v>767</v>
       </c>
       <c r="D7" t="n">
-        <v>1881</v>
+        <v>1157</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>2023</v>
+        <v>2032</v>
       </c>
       <c r="G7" t="n">
-        <v>2819</v>
+        <v>2828</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>3289</v>
+        <v>3298</v>
       </c>
       <c r="J7" t="n">
-        <v>3687</v>
+        <v>3696</v>
       </c>
       <c r="K7" t="n">
         <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>3687</v>
+        <v>3696</v>
       </c>
       <c r="M7" t="n">
-        <v>3858</v>
+        <v>3867</v>
       </c>
     </row>
     <row r="8">
@@ -767,19 +767,19 @@
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>2132</v>
+        <v>2169</v>
       </c>
       <c r="J8" t="n">
-        <v>2718</v>
+        <v>2755</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>2718</v>
+        <v>2755</v>
       </c>
       <c r="M8" t="n">
-        <v>3106</v>
+        <v>3143</v>
       </c>
     </row>
     <row r="9">
@@ -790,10 +790,10 @@
         <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>1389</v>
+        <v>1157</v>
       </c>
       <c r="D9" t="n">
-        <v>2076</v>
+        <v>1844</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -849,19 +849,19 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="J10" t="n">
-        <v>1952</v>
+        <v>1953</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
       </c>
       <c r="L10" t="n">
-        <v>1952</v>
+        <v>1953</v>
       </c>
       <c r="M10" t="n">
-        <v>2433</v>
+        <v>2434</v>
       </c>
     </row>
     <row r="11">
@@ -890,19 +890,19 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="J11" t="n">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
       </c>
       <c r="L11" t="n">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="M11" t="n">
-        <v>1740</v>
+        <v>1741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>